<commit_message>
chore(audit): drop zero-qty placeholder rows from off-master sheet
Raw inventory files sometimes include placeholder rows with qty=0 (new
product SKUs registered but no stock yet, deprecated SKUs lingering in
the export).  These don't represent invisible inventory and don't need
master entries.  Filter them out of the off_master_asins sheet so the
audit shows only ASINs where real units are being silently dropped.

Off-master count drops from 77 → 37 on current data: 5 Nexlev (the
FBA80078-80082 family with 50 units total) + 32 Fossil tail SKUs.
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -2155,7 +2155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2193,40 +2193,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B0FN4GJ9S1</t>
+          <t>B07LDJJ4JP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FBK79790</t>
+          <t>FBA72564</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>white mulberry</t>
+          <t>fossil</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ampm</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>715</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B07LDJJ4JP</t>
+          <t>B07RMH1BMS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FBA72564</t>
+          <t>FBA72563</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2243,18 +2243,18 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>159</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B07RMH1BMS</t>
+          <t>B07LDHVWTF</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FBA72563</t>
+          <t>FBA72562</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2271,18 +2271,18 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>103</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B07LDHVWTF</t>
+          <t>B07S3X9JYX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FBA72562</t>
+          <t>FBA72570</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2299,18 +2299,18 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B07S3X9JYX</t>
+          <t>B07RMH1F26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FBA72570</t>
+          <t>FBA72907</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2327,18 +2327,18 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B0GQCB4PJC</t>
+          <t>B0GQGZVGLL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FBA80079</t>
+          <t>FBA80082</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2361,12 +2361,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B0GQGK4GJ7</t>
+          <t>B0GQC12GDP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FBA80081</t>
+          <t>FBA80078</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2389,12 +2389,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B0GQGXR9D7</t>
+          <t>B0GQGK4GJ7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FBA80080</t>
+          <t>FBA80081</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2417,12 +2417,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B0GQGZVGLL</t>
+          <t>B0GQCB4PJC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FBA80082</t>
+          <t>FBA80079</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2445,17 +2445,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B07RMH1F26</t>
+          <t>B0GQGXR9D7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FBA72907</t>
+          <t>FBA80080</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>fossil</t>
+          <t>nexlev</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>10</v>
@@ -2473,17 +2473,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>B0GQC12GDP</t>
+          <t>B00STAYV6C</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FBA80078</t>
+          <t>FBS66968</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>nexlev</t>
+          <t>fossil</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2495,18 +2495,18 @@
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>B00STAYV6C</t>
+          <t>B0DKJJDZSF</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FBS66968</t>
+          <t>FBS79626</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2520,21 +2520,21 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B085YFCGNF</t>
+          <t>B07RPQWF6B</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FBA74027</t>
+          <t>FBP75458</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
         <v>4</v>
@@ -2585,12 +2585,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B0DKJJDZSF</t>
+          <t>B07SPCV89W</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FBS79626</t>
+          <t>FBA72904</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>4</v>
@@ -2613,12 +2613,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>B07RPQWF6B</t>
+          <t>B085YFCGNF</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FBP75458</t>
+          <t>FBA74027</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>4</v>
@@ -2641,12 +2641,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B07SPCV89W</t>
+          <t>B00DUCIUDY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FBA72904</t>
+          <t>FBO70542</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2660,21 +2660,21 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B00DUCIUDY</t>
+          <t>B0DKJG6R31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FBO70542</t>
+          <t>FBS79623</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2697,12 +2697,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B0DKJG6R31</t>
+          <t>B07N6KCJM4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FBS79623</t>
+          <t>FBA72566</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2716,7 +2716,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>3</v>
@@ -2725,12 +2725,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B07N6KCJM4</t>
+          <t>B00VATDB10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FBA72566</t>
+          <t>FBN69542</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2744,21 +2744,21 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>B00VATDB10</t>
+          <t>B0BQZGJHKV</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FBN69542</t>
+          <t>FBS77967</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2772,7 +2772,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>2</v>
@@ -2781,12 +2781,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>B0BQZGJHKV</t>
+          <t>B08K969L6V</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FBS77967</t>
+          <t>FBK74025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2800,7 +2800,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>2</v>
@@ -2893,12 +2893,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B08K969L6V</t>
+          <t>B00Z52HG6O</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FBK74025</t>
+          <t>FBO77065</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2912,21 +2912,21 @@
         </is>
       </c>
       <c r="E27" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" t="n">
         <v>1</v>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>B01MZWUN47</t>
+          <t>B00DH9NPBM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FBK72029</t>
+          <t>FBO66628</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2949,12 +2949,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B00DH9NPBM</t>
+          <t>B01MZWUN47</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>FBO66628</t>
+          <t>FBK72029</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2977,12 +2977,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B00Z52HG6O</t>
+          <t>B088NYP2LX</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FBO77065</t>
+          <t>FBA78457</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>1</v>
@@ -3005,12 +3005,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B0CZSFTY4V</t>
+          <t>B088NZCC28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>FBS79431</t>
+          <t>FBA78458</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3024,7 +3024,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>1</v>
@@ -3033,12 +3033,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B088NZCC28</t>
+          <t>B0DKJJBBTS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>FBA78458</t>
+          <t>FBA79620</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3052,7 +3052,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
@@ -3061,12 +3061,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>B088NYP2LX</t>
+          <t>B0CZSFTY4V</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>FBA78457</t>
+          <t>FBS79431</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3080,7 +3080,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -3117,12 +3117,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>B0DSBQL4PK</t>
+          <t>B0CQNSQ9BJ</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>FBA79747</t>
+          <t>FBA79250</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3136,7 +3136,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
         <v>1</v>
@@ -3145,12 +3145,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>B0DKJJBBTS</t>
+          <t>B0DJ2XK4NR</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FBA79620</t>
+          <t>FBS79646</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
@@ -3173,12 +3173,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>B0CQNSQ9BJ</t>
+          <t>B0FTKJC5JW</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FBA79250</t>
+          <t>FBA79936</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3192,7 +3192,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
@@ -3201,12 +3201,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>B0DJ2XK4NR</t>
+          <t>B0DSBQL4PK</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>FBS79646</t>
+          <t>FBA79747</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3220,1130 +3220,10 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
         <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>B0FTKJC5JW</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>FBA79936</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>B074ZHN54C</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>FBN66667</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>2</v>
-      </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>B00KNK7UHI</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>FBS76475</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>B079HF6BL3</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>FBO69618</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>B07T53XXCF</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>FBA79149</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>2</v>
-      </c>
-      <c r="F43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>B094R8FJ6J</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>FBS79559</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>B09876MGQ1</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>FBO74936</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>B07SRVV8V4</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>FBA71998</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>B0CJ6ZW8FP</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>FBA79141</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>2</v>
-      </c>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>B0CFH5R7Y7</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>FBA79002</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>B0CFH2C369</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>FBA79001</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>4</v>
-      </c>
-      <c r="F49" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>B0CFH2B2MV</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>FBA79000</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>4</v>
-      </c>
-      <c r="F50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>B0CFFQK45G</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>FBA78999</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>4</v>
-      </c>
-      <c r="F51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>B0CCHNK41V</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>FBA79044</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>2</v>
-      </c>
-      <c r="F52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>B0CCHMD6QH</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>FBA79047</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>2</v>
-      </c>
-      <c r="F53" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>B0CCHGLV6Y</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>FBA79051</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>2</v>
-      </c>
-      <c r="F54" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>B0C7WLLHPG</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>FBA79036</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>2</v>
-      </c>
-      <c r="F55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>B0C77PP76Y</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>FBA79020</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>2</v>
-      </c>
-      <c r="F56" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>B0BSHTX51F</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>FBA79220</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>2</v>
-      </c>
-      <c r="F57" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>B0BLK9QL7X</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>FBA76731</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>3</v>
-      </c>
-      <c r="F58" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>B0BLJYX15C</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>FBA76709</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>3</v>
-      </c>
-      <c r="F59" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>B0BLK1Z7PJ</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>FBA76713</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>ampm</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>3</v>
-      </c>
-      <c r="F60" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>B0BHCJHWCL</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>FBO76786</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>2</v>
-      </c>
-      <c r="F61" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>B0BFZHWXBM</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>FBA76896</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>2</v>
-      </c>
-      <c r="F62" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>B07T2XZ5K4</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>FBA79802</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>2</v>
-      </c>
-      <c r="F63" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>B0D956WQVM</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>FBS79543</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E64" t="n">
-        <v>2</v>
-      </c>
-      <c r="F64" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>B0DJ2VY8GL</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>FBS79648</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>2</v>
-      </c>
-      <c r="F65" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>B0D9568SNM</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>FBS79560</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E66" t="n">
-        <v>2</v>
-      </c>
-      <c r="F66" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>B0D9361BZL</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>FBS79535</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>2</v>
-      </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>B0CZSDZ5V1</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>FBA79420</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E68" t="n">
-        <v>2</v>
-      </c>
-      <c r="F68" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>B0D9536B5Z</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>FBS79546</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E69" t="n">
-        <v>2</v>
-      </c>
-      <c r="F69" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>B0D936GDTN</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>FBS79536</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>2</v>
-      </c>
-      <c r="F70" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>B0FM3LBN87</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>FBK79595</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>B0F99VFBGY</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>FBK79685</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E72" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>B0F2MZJH82</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>FBA79987</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>B0DT37Y5FY</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>FBA79902</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>2</v>
-      </c>
-      <c r="F74" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>B0DSBT6FW8</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>FBA79734</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>2</v>
-      </c>
-      <c r="F75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>B0DSBR61QS</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>FBA79901</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E76" t="n">
-        <v>2</v>
-      </c>
-      <c r="F76" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>B0DSBPRB2W</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>FBA79739</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>2</v>
-      </c>
-      <c r="F77" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>B0FRVT4SJ1</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>FBA79922</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>fossil</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="E78" t="n">
-        <v>2</v>
-      </c>
-      <c r="F78" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: refresh business_ads_joined with Model-from-master applied to 548 ASINs
Deployed business_ads_joined.csv was stale — it predated today's
Model-from-master fix in step4 (b174084).  548 Nexlev / WM / AA
ASINs that have a Model in sku_master but no Model in their
business_report row were landing in the model=NaN bucket,
inflating AMS Trend's phantom "(no model)" GMV by Rs 25.6L and
firing Check 19 fail-loud on 3 (brand, NaN-model) buckets.

After a fresh step4 + step5 run with the fix in place: every
admissible ASIN resolves to its master Model.  Test case
B0CDPMX152 (Nexlev GS-02 Steam Iron) — was model=NaN across
W21-W24, now model="GS-02" across all four weeks.

Audit final:
  0 fail-loud, 93 informational
  Check 19 (per-model AMS > Sales drift): 0
  Cross-route checks 12-17: all 0

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1_raw_vs_snapshot" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_snapshot_vs_route" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_never_zero" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_channel_case_drift" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5_went_to_zero" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6_master_completeness" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7_brand_name_consistency" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8_latest_week_presence" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="9_brand_retags_info" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10_off_master_asins" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="11_raw_vs_snap_sales" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="12_cross_route_inv" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="13_cross_route_sales" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="14_cross_route_ads" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="15_cross_route_sessions" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="16_cross_route_units" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="17_cross_route_brands" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="18_off_master_sales" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="19_ams_gt_sales_per_model" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_raw_vs_snapshot" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_snapshot_vs_route" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_never_zero" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_channel_case_drift" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_went_to_zero" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_master_completeness" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_brand_name_consistency" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_latest_week_presence" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_brand_retags_info" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_off_master_asins" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_raw_vs_snap_sales" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_cross_route_inv" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_cross_route_sales" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_cross_route_ads" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_cross_route_sessions" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_cross_route_units" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_cross_route_brands" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_off_master_sales" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_ams_gt_sales_per_model" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,13 +35,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,7 +55,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,12 +63,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,32 +447,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>week_num</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>raw_units</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>snap_units</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -697,32 +709,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>asin</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>raw_sku</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>brand_folder</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>weeks_seen</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>total_qty</t>
         </is>
@@ -771,7 +783,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -799,7 +811,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -827,7 +839,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -855,7 +867,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -883,7 +895,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -911,7 +923,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -939,7 +951,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -963,21 +975,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>note</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>asin</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>raw_sku</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>brand_folder</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>weeks_seen</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>total_units</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>clean — (info) Off-master ASINs in raw sales</t>
-        </is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FBA79347</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>other_channels</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pharmaeasy</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -995,7 +1063,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1023,32 +1091,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>layer</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>week_num</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>snap_units</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>route_units</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1117,7 +1185,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1145,7 +1213,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1173,32 +1241,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>layer</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>prior_3wk</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>latest</t>
         </is>
@@ -1303,22 +1371,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>issue</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>asin</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
@@ -1589,7 +1657,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1613,26 +1681,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>layer</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>brand</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>week</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1641,160 +1694,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for audio array in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for nexlev in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>tonor</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for tonor in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>white mulberry</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>24</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for white mulberry in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>24</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for audio array in inventory for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>24</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for nexlev in inventory for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>tonor</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>24</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for tonor in inventory for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>white mulberry</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>24</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for white mulberry in inventory for W24</t>
+          <t>clean — Brand missing from a layer (diagnostic)</t>
         </is>
       </c>
     </row>
@@ -1813,32 +1713,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>week_num</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>raw_units</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>snap_units</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>

</xml_diff>

<commit_message>
data: W24 inventory snapshots refreshed (operator manual update)
Operator pushed updated Inventory Snapshot.xlsx for all 4 tracked
brands (AA / Nexlev / Tonor / WM).  Re-ran inv_model + inv_snap +
margin + returns + inbound + audit.

W24 inventory totals (all channels combined):
  Audio Array     76,895 units  Rs 12.03 Cr
  Nexlev          75,156 units  Rs  6.97 Cr
  White Mulberry   8,620 units  Rs  0.83 Cr
  Tonor            3,660 units  Rs  0.41 Cr

Pipeline integrity audit: 0 fail-loud, 94 informational.
Cross-route inventory check (#12) = 0 drift.
All cross-route checks (12-17 + 19) clean.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -1132,10 +1132,10 @@
         <v>24</v>
       </c>
       <c r="C2" t="n">
-        <v>165783</v>
+        <v>164331</v>
       </c>
       <c r="D2" t="n">
-        <v>165783</v>
+        <v>164331</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1156,10 +1156,10 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>153377</v>
+        <v>151925</v>
       </c>
       <c r="D3" t="n">
-        <v>153377</v>
+        <v>151925</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1237,7 +1237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1303,26 +1303,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sales</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>audio array</t>
+          <t>white mulberry</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bi worldwide</t>
+          <t>pipeline</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>units_sold</t>
+          <t>inventory_units</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1500</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -1336,23 +1336,51 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bi worldwide</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>units_sold</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>nexlev</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>bi worldwide</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>units_sold</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E5" t="n">
         <v>13</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: refresh AMS aggregates to align with re-derived sales
After re-running sales_auto_etl during the W23 regression investigation,
business_ads_joined was stale relative to weekly_sales_snapshot, causing
Check 19 to flag 3 NaN-model rows again.  Full chain re-run
(business_report_derive → biz_ads → step3 → step4 → step5) brings them
back into alignment.

Final audit:
  0 fail-loud, 94 informational
  Check 19 (per-model AMS > Sales drift): 0
  Cross-route checks 12-17: all 0

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1_raw_vs_snapshot" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_snapshot_vs_route" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_never_zero" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_channel_case_drift" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5_went_to_zero" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6_master_completeness" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7_brand_name_consistency" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8_latest_week_presence" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="9_brand_retags_info" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10_off_master_asins" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="11_raw_vs_snap_sales" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="12_cross_route_inv" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="13_cross_route_sales" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="14_cross_route_ads" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="15_cross_route_sessions" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="16_cross_route_units" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="17_cross_route_brands" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="18_off_master_sales" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="19_ams_gt_sales_per_model" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_raw_vs_snapshot" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_snapshot_vs_route" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_never_zero" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_channel_case_drift" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_went_to_zero" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_master_completeness" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_brand_name_consistency" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_latest_week_presence" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_brand_retags_info" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_off_master_asins" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_raw_vs_snap_sales" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_cross_route_inv" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_cross_route_sales" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_cross_route_ads" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_cross_route_sessions" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_cross_route_units" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_cross_route_brands" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_off_master_sales" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_ams_gt_sales_per_model" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35,13 +35,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,7 +55,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,12 +63,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,32 +447,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>week_num</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>raw_units</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>snap_units</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -697,32 +709,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>asin</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>raw_sku</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>brand_folder</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>weeks_seen</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>total_qty</t>
         </is>
@@ -771,7 +783,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -799,7 +811,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -827,7 +839,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -855,7 +867,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -883,7 +895,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -911,7 +923,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -939,7 +951,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -963,21 +975,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>note</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>asin</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>raw_sku</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>brand_folder</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>weeks_seen</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>total_units</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>clean — (info) Off-master ASINs in raw sales</t>
-        </is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FBA79347</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>other_channels</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pharmaeasy</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -995,7 +1063,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1023,32 +1091,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>layer</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>week_num</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>snap_units</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>route_units</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1117,7 +1185,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1145,7 +1213,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1173,32 +1241,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>layer</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>prior_3wk</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>latest</t>
         </is>
@@ -1331,22 +1399,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>issue</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>asin</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
@@ -1617,7 +1685,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1641,26 +1709,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>layer</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>brand</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>week</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1669,160 +1722,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for audio array in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for nexlev in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>tonor</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for tonor in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>white mulberry</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>24</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for white mulberry in sales for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>24</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for audio array in inventory for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>nexlev</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>24</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for nexlev in inventory for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>tonor</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>24</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for tonor in inventory for W24</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>inventory</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>white mulberry</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>24</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MISSING — no rows for white mulberry in inventory for W24</t>
+          <t>clean — Brand missing from a layer (diagnostic)</t>
         </is>
       </c>
     </row>
@@ -1841,32 +1741,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>week_num</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>raw_units</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>snap_units</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>delta</t>
         </is>

</xml_diff>

<commit_message>
data: W26 add Flipkart channel to Audio Array other_channels
Operator updated data/raw/sales/Week 26/Audio_Array/other_channels.xlsx
to include the Flipkart channel rows (previously missing from W26).
Re-ran sales_auto_etl + business_ads chain + integrity audit.

Sales effect (W26 weekly_sales_snapshot row count 283 → 340):
  Flipkart   57 SKU-rows  42 units   (new channel for W26)

Audit: clean (0 fail-louds, 128 info rows).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -1704,7 +1704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1943,12 +1943,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>audio array</t>
+          <t>nexlev</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>38</v>
+        <v>2056</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>nexlev</t>
+          <t>tonor</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2056</v>
+        <v>27</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tonor</t>
+          <t>white mulberry</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>27</v>
+        <v>638</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>b2b</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2041,37 +2041,9 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>638</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>sales</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>white mulberry</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>b2b</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>units_sold</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ci(weekly-sync): shorten Vendor Returns pull 90d -> 30d
At 90 days / 14-day chunks the step was running ~60 min alone (14
chunks × ~4 min each), which pushed run 28771958674 past the 120-min
timeout mid-chunk without touching any downstream ETL.

30d = 3 chunks × 2 vendor accounts ≈ 25 min.  Historic 90d window still
available via `python scripts/sp_vendor_returns_pull.py --days 90` for
manual reconciliation.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -31,6 +31,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22_category_coverage" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23_sp_api_ingestion" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_ams_vs_sales_brand" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25_inv_snapshot_freshness" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26_pit_snapshot_freshness" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,30 +746,6 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>EXTRA IN SNAPSHOT (stale rows?)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>26</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>pipeline</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>40427</v>
-      </c>
-      <c r="D13" t="n">
-        <v>39427</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>UNITS MISMATCH (silent drop)</t>
         </is>
       </c>
     </row>
@@ -4805,10 +4783,10 @@
         <v>26</v>
       </c>
       <c r="C2" t="n">
-        <v>179341</v>
+        <v>180341</v>
       </c>
       <c r="D2" t="n">
-        <v>179341</v>
+        <v>180341</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -4829,10 +4807,10 @@
         <v>26</v>
       </c>
       <c r="C3" t="n">
-        <v>171380</v>
+        <v>172380</v>
       </c>
       <c r="D3" t="n">
-        <v>171380</v>
+        <v>172380</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -4988,6 +4966,150 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>clean — Inventory snapshot behind latest raw week (silent ETL failure)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>anchor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>lag_hours</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>data\processed\returns_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>data\processed\inventory_model_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>snapshot older than anchor by &gt;24h — ETL likely failed silently on the last cron run</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>data\processed\margin_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>data\processed\inventory_model_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>snapshot older than anchor by &gt;24h — ETL likely failed silently on the last cron run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>data\processed\inbound_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>data\processed\inventory_model_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>snapshot older than anchor by &gt;24h — ETL likely failed silently on the last cron run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>data\processed\reviews_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>data\processed\inventory_model_snapshot.csv</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>snapshot older than anchor by &gt;24h — ETL likely failed silently on the last cron run</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5098,7 +5220,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>open order</t>
+          <t>pipeline</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5107,7 +5229,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>240</v>
+        <v>572</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -5126,7 +5248,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>open order</t>
+          <t>pipeline</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5135,7 +5257,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>6000</v>
+        <v>500</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -5180,7 +5302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5436,7 +5558,7 @@
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>FBA74928</t>
+          <t>FBA80105</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -5450,10 +5572,24 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
+          <t>FBA74928</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DUPLICATE SKU (2× in master)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5522,7 +5658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7333,30 +7469,6 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>26</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>audio array</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>pipeline</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>26295</v>
-      </c>
-      <c r="E76" t="n">
-        <v>25295</v>
-      </c>
-      <c r="F76" t="n">
-        <v>-1000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
audit(check 27): all-weeks AMS Trend vs Sales Trend brand cross-check
Companion to Check 24 that covers ALL weeks, not just latest_week.
Would have caught the 2026-07-13 AA-over-count / Fossil-mistag bug at
commit-1 instead of hiding for 4 weeks.

Tolerance intentionally looser than Check 24 (Rs 10K AND >= 2%
relative; both must fire) so it doesn't flag legitimate small drifts
in older weeks that predate SP-API 1P ingest coverage.

Post-fix baseline: 55 legitimate historical-coverage-gap drifts on
W4-W13 (SP-API 1P scope narrower than raw sales scope in those weeks).
Any NEW drift on a recent week is a real regression to investigate.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -33,6 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_ams_vs_sales_brand" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25_inv_snapshot_freshness" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26_pit_snapshot_freshness" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27_ams_vs_sales_brand_history" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5259,7 +5260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5287,38 +5288,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>data\ams_weekly_data\processed_ads\business_ads_joined.csv</t>
+          <t>data\processed\inventory_model_snapshot.csv</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>data\ams_weekly_data\ams_weekly_fact\ams_weekly_fact_with_category.csv</t>
+          <t>data\processed\inventory_ams_snapshot.csv</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4934.1</v>
+        <v>253831.6</v>
       </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>business_ads_joined → ams_weekly_fact_with_category (step5 needs re-run)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>data\processed\inventory_model_snapshot.csv</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>data\processed\inventory_ams_snapshot.csv</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>253831.6</v>
-      </c>
-      <c r="D3" t="inlineStr">
         <is>
           <t>inventory_model_snapshot → inventory_ams_snapshot (inv_snap needs re-run)</t>
         </is>
@@ -5335,7 +5316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5373,50 +5354,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Audio Array</t>
+          <t>Nexlev</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sessions</t>
+          <t>attributed</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>129946</v>
+        <v>1719322</v>
       </c>
       <c r="D2" t="n">
-        <v>316756</v>
+        <v>751045</v>
       </c>
       <c r="E2" t="n">
-        <v>-59</v>
+        <v>128.9</v>
       </c>
       <c r="F2" t="inlineStr">
-        <is>
-          <t>DROP &gt; 50% vs prior 4-week median</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Nexlev</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>attributed</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1719322</v>
-      </c>
-      <c r="D3" t="n">
-        <v>751045</v>
-      </c>
-      <c r="E3" t="n">
-        <v>128.9</v>
-      </c>
-      <c r="F3" t="inlineStr">
         <is>
           <t>SPIKE &gt; 2x vs prior 4-week median</t>
         </is>
@@ -5710,6 +5665,1652 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>week</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>sales_trend_amz_side</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ams_trend_gmv</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>delta_rs</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>delta_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3095009.71</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-3095009.71</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2392739.69</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-2392739.69</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>324781.32</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-324781.32</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1906527.52</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-1906527.52</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2654996.45</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-2654996.45</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1396572.19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-1396572.19</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>346045.54</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-346045.54</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1115446.59</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-1115446.59</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3119828.81</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-3119828.81</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1608376.27</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-1608376.27</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>314639.94</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-314639.94</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1136712.62</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-1136712.62</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3039578.87</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-3039578.87</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1577064.99</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-1577064.99</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>252253.44</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-252253.44</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1072173.2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-1072173.2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3033347.93</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-3033347.93</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1410246.25</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-1410246.25</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>203072.94</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-203072.94</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>942950.09</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-942950.09</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2957495.02</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-2957495.02</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1467359.63</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-1467359.63</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>184894.03</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-184894.03</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1185369.31</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-1185369.31</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3066258.52</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-3066258.52</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1643099.86</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-1643099.86</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>110584.75</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-110584.75</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>914785.01</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-914785.01</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3097839.36</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-3097839.36</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2190479.57</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-2190479.57</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>87927.05</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-87927.05</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>667998.22</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-667998.22</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2904810.42</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-2904810.42</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1929190.89</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-1929190.89</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>114738.08</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-114738.08</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>555963.54</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>-555963.54</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3225192.62</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-3225192.62</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1573750.55</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-1573750.55</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>161457.56</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-161457.56</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>784099.59</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-784099.59</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>3058255.43</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-3058255.43</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1694388.76</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-1694388.76</v>
+      </c>
+      <c r="F43" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>114756.74</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-114756.74</v>
+      </c>
+      <c r="F44" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>663401.58</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-663401.58</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2511216.45</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-2511216.45</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1917524.41</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-1917524.41</v>
+      </c>
+      <c r="F47" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>151414.35</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-151414.35</v>
+      </c>
+      <c r="F48" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>494952.2</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>-494952.2</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-100</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>W16</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>470608.43</v>
+      </c>
+      <c r="D50" t="n">
+        <v>386716.9</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-83891.53</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-17.83</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>W18</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>667942.12</v>
+      </c>
+      <c r="D51" t="n">
+        <v>584995.51</v>
+      </c>
+      <c r="E51" t="n">
+        <v>-82946.61</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-12.42</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>W19</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>713759.26</v>
+      </c>
+      <c r="D52" t="n">
+        <v>690287.23</v>
+      </c>
+      <c r="E52" t="n">
+        <v>-23472.03</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-3.29</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>W20</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1077787.08</v>
+      </c>
+      <c r="D53" t="n">
+        <v>976121.8199999999</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-101665.26</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-9.43</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>W21</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>911351.88</v>
+      </c>
+      <c r="D54" t="n">
+        <v>749514.71</v>
+      </c>
+      <c r="E54" t="n">
+        <v>-161837.17</v>
+      </c>
+      <c r="F54" t="n">
+        <v>-17.76</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>W22</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>888714.46</v>
+      </c>
+      <c r="D55" t="n">
+        <v>823641.58</v>
+      </c>
+      <c r="E55" t="n">
+        <v>-65072.88</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-7.32</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>W23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1135238.81</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1078365.93</v>
+      </c>
+      <c r="E56" t="n">
+        <v>-56872.88</v>
+      </c>
+      <c r="F56" t="n">
+        <v>-5.01</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-08-02
</commit_message>
<xml_diff>
--- a/data/processed/pipeline_integrity_audit.xlsx
+++ b/data/processed/pipeline_integrity_audit.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,6 +615,30 @@
         <v>14876</v>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>EXTRA IN SNAPSHOT (stale rows?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13951</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13951</v>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>EXTRA IN SNAPSHOT (stale rows?)</t>
         </is>
@@ -715,12 +739,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>asin</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sales_trend_amzn+1p_gmv</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ams_trend_gmv</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>delta_rs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -728,7 +772,147 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>clean — Cross-source sales drift (diagnostic)</t>
+          <t>B0DB5VG39T</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>186372.8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>186372.8</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B0DB5VVPSB</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>44735.59</v>
+      </c>
+      <c r="C3" t="n">
+        <v>66594.91</v>
+      </c>
+      <c r="D3" t="n">
+        <v>21859.32</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B0DB5W4TCP</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1481.36</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9866.120000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8384.76</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B0DB5YTQZV</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7454.24</v>
+      </c>
+      <c r="C5" t="n">
+        <v>48111.84</v>
+      </c>
+      <c r="D5" t="n">
+        <v>40657.6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B0DP2VVRND</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8894.07</v>
+      </c>
+      <c r="C6" t="n">
+        <v>122396.47</v>
+      </c>
+      <c r="D6" t="n">
+        <v>113502.4</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B0DP3194QN</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3143.22</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6108.47</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2965.25</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B0DP32F346</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>70909.37</v>
+      </c>
+      <c r="D8" t="n">
+        <v>70909.37</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AMAZON+1P GMV drifts between sales_snapshot and business_ads_joined</t>
         </is>
       </c>
     </row>
@@ -799,12 +983,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>asin</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sales_trend_units</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ams_trend_units</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -812,7 +1016,126 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>clean — Cross-source units drift (diagnostic)</t>
+          <t>B0DB5VG39T</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AMAZON+1P UNITS drift between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B0DB5VVPSB</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C3" t="n">
+        <v>19</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AMAZON+1P UNITS drift between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B0DB5W4TCP</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AMAZON+1P UNITS drift between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B0DB5YTQZV</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" t="n">
+        <v>24</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AMAZON+1P UNITS drift between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B0DP2VVRND</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>72</v>
+      </c>
+      <c r="D6" t="n">
+        <v>67</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AMAZON+1P UNITS drift between sales_snapshot and business_ads_joined</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B0DP32F346</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>27</v>
+      </c>
+      <c r="D7" t="n">
+        <v>27</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AMAZON+1P UNITS drift between sales_snapshot and business_ads_joined</t>
         </is>
       </c>
     </row>
@@ -925,7 +1248,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -938,21 +1261,21 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2414</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>121227</v>
+        <v>186373</v>
       </c>
       <c r="F2" t="n">
-        <v>118813</v>
+        <v>186373</v>
       </c>
       <c r="G2" t="n">
-        <v>4921</v>
+        <v>18637280</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -965,21 +1288,21 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>32187</v>
+        <v>8894</v>
       </c>
       <c r="E3" t="n">
-        <v>120203</v>
+        <v>122396</v>
       </c>
       <c r="F3" t="n">
-        <v>88015</v>
+        <v>113502</v>
       </c>
       <c r="G3" t="n">
-        <v>273.4</v>
+        <v>1276.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -995,18 +1318,18 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>57778</v>
+        <v>70909</v>
       </c>
       <c r="F4" t="n">
-        <v>57778</v>
+        <v>70909</v>
       </c>
       <c r="G4" t="n">
-        <v>5777803</v>
+        <v>7090937</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1019,21 +1342,21 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1864</v>
+        <v>7454</v>
       </c>
       <c r="E5" t="n">
-        <v>50991</v>
+        <v>48112</v>
       </c>
       <c r="F5" t="n">
-        <v>49128</v>
+        <v>40658</v>
       </c>
       <c r="G5" t="n">
-        <v>2636.2</v>
+        <v>545.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1046,21 +1369,21 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11184</v>
+        <v>44736</v>
       </c>
       <c r="E6" t="n">
-        <v>40330</v>
+        <v>66595</v>
       </c>
       <c r="F6" t="n">
-        <v>29146</v>
+        <v>21859</v>
       </c>
       <c r="G6" t="n">
-        <v>260.6</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1073,16 +1396,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1481</v>
       </c>
       <c r="E7" t="n">
-        <v>5590</v>
+        <v>9866</v>
       </c>
       <c r="F7" t="n">
-        <v>5590</v>
+        <v>8385</v>
       </c>
       <c r="G7" t="n">
-        <v>558984</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -1138,13 +1461,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C2" t="n">
-        <v>184763</v>
+        <v>181896</v>
       </c>
       <c r="D2" t="n">
-        <v>184763</v>
+        <v>181896</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1162,13 +1485,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" t="n">
-        <v>177534</v>
+        <v>174472</v>
       </c>
       <c r="D3" t="n">
-        <v>177534</v>
+        <v>174472</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1302,12 +1625,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sales_trend_amz_side</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ams_trend_gmv</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>delta_rs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -1315,7 +1658,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>clean — AMS Trend GMV vs Sales Trend Amazon-side per brand</t>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>538616.98</v>
+      </c>
+      <c r="C2" t="n">
+        <v>983268.48</v>
+      </c>
+      <c r="D2" t="n">
+        <v>444651.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AMS Trend GMV ≠ Sales Trend Amazon-side gross_sales — one chain is missing a 3P/1P source or column format</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1429,25 +1786,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tonor</t>
+          <t>white mulberry</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>171494.05</v>
+        <v>1077787.08</v>
       </c>
       <c r="D2" t="n">
-        <v>161455.91</v>
+        <v>971121.8199999999</v>
       </c>
       <c r="E2" t="n">
-        <v>-10038.14</v>
+        <v>-106665.26</v>
       </c>
       <c r="F2" t="n">
-        <v>-5.85</v>
+        <v>-9.9</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -1458,7 +1815,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1467,16 +1824,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>713759.26</v>
+        <v>911351.88</v>
       </c>
       <c r="D3" t="n">
-        <v>676492.3199999999</v>
+        <v>732132.51</v>
       </c>
       <c r="E3" t="n">
-        <v>-37266.94</v>
+        <v>-179219.37</v>
       </c>
       <c r="F3" t="n">
-        <v>-5.22</v>
+        <v>-19.67</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -1487,7 +1844,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1496,16 +1853,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1077787.08</v>
+        <v>888714.46</v>
       </c>
       <c r="D4" t="n">
-        <v>971121.8199999999</v>
+        <v>732317.85</v>
       </c>
       <c r="E4" t="n">
-        <v>-106665.26</v>
+        <v>-156396.61</v>
       </c>
       <c r="F4" t="n">
-        <v>-9.9</v>
+        <v>-17.6</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1516,7 +1873,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>W21</t>
+          <t>W23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1525,16 +1882,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>911351.88</v>
+        <v>1135238.81</v>
       </c>
       <c r="D5" t="n">
-        <v>732132.51</v>
+        <v>1031959.15</v>
       </c>
       <c r="E5" t="n">
-        <v>-179219.37</v>
+        <v>-103279.66</v>
       </c>
       <c r="F5" t="n">
-        <v>-19.67</v>
+        <v>-9.1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1545,7 +1902,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>W22</t>
+          <t>W24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1554,16 +1911,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>888714.46</v>
+        <v>624059.3199999999</v>
       </c>
       <c r="D6" t="n">
-        <v>732317.85</v>
+        <v>699655.0600000001</v>
       </c>
       <c r="E6" t="n">
-        <v>-156396.61</v>
+        <v>75595.74000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>-17.6</v>
+        <v>12.11</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1574,7 +1931,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>W23</t>
+          <t>W25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1583,16 +1940,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1135238.81</v>
+        <v>970911.86</v>
       </c>
       <c r="D7" t="n">
-        <v>1031959.15</v>
+        <v>907348.3</v>
       </c>
       <c r="E7" t="n">
-        <v>-103279.66</v>
+        <v>-63563.56</v>
       </c>
       <c r="F7" t="n">
-        <v>-9.1</v>
+        <v>-6.55</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1603,25 +1960,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>W24</t>
+          <t>W26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>white mulberry</t>
+          <t>tonor</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>624059.3199999999</v>
+        <v>199271.08</v>
       </c>
       <c r="D8" t="n">
-        <v>699655.0600000001</v>
+        <v>181904.13</v>
       </c>
       <c r="E8" t="n">
-        <v>75595.74000000001</v>
+        <v>-17366.95</v>
       </c>
       <c r="F8" t="n">
-        <v>12.11</v>
+        <v>-8.720000000000001</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1632,7 +1989,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>W25</t>
+          <t>W26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1641,16 +1998,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>970911.86</v>
+        <v>768346.55</v>
       </c>
       <c r="D9" t="n">
-        <v>907348.3</v>
+        <v>704910.12</v>
       </c>
       <c r="E9" t="n">
-        <v>-63563.56</v>
+        <v>-63436.43</v>
       </c>
       <c r="F9" t="n">
-        <v>-6.55</v>
+        <v>-8.26</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1661,25 +2018,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>W26</t>
+          <t>W27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tonor</t>
+          <t>white mulberry</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>199271.08</v>
+        <v>1122800.58</v>
       </c>
       <c r="D10" t="n">
-        <v>181904.13</v>
+        <v>1090799.74</v>
       </c>
       <c r="E10" t="n">
-        <v>-17366.95</v>
+        <v>-32000.84</v>
       </c>
       <c r="F10" t="n">
-        <v>-8.720000000000001</v>
+        <v>-2.85</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1690,7 +2047,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>W26</t>
+          <t>W28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1699,16 +2056,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>768346.55</v>
+        <v>1192822.95</v>
       </c>
       <c r="D11" t="n">
-        <v>704910.12</v>
+        <v>1167062.78</v>
       </c>
       <c r="E11" t="n">
-        <v>-63436.43</v>
+        <v>-25760.17</v>
       </c>
       <c r="F11" t="n">
-        <v>-8.26</v>
+        <v>-2.16</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1719,7 +2076,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>W27</t>
+          <t>W31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1728,76 +2085,18 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1122800.58</v>
+        <v>538616.98</v>
       </c>
       <c r="D12" t="n">
-        <v>1090799.74</v>
+        <v>983268.48</v>
       </c>
       <c r="E12" t="n">
-        <v>-32000.84</v>
+        <v>444651.5</v>
       </c>
       <c r="F12" t="n">
-        <v>-2.85</v>
+        <v>82.55</v>
       </c>
       <c r="G12" t="inlineStr">
-        <is>
-          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>W28</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>tonor</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>312502.37</v>
-      </c>
-      <c r="D13" t="n">
-        <v>300387.97</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-12114.4</v>
-      </c>
-      <c r="F13" t="n">
-        <v>-3.88</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>W28</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>white mulberry</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1192822.95</v>
-      </c>
-      <c r="D14" t="n">
-        <v>1167062.78</v>
-      </c>
-      <c r="E14" t="n">
-        <v>-25760.17</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-2.16</v>
-      </c>
-      <c r="G14" t="inlineStr">
         <is>
           <t>AMS Trend brand-week GMV drifts from Sales Trend Amazon+1P &gt;= 2% AND &gt;= Rs 10,000 — possible brand mis-tag (see Fossil-to-AA pattern of 2026-07-13) OR missing/duplicate source ingest for this brand-week</t>
         </is>
@@ -1926,7 +2225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1964,26 +2263,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>sales</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>white mulberry</t>
+          <t>audio array</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>open order</t>
+          <t>flipkart</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>inventory_units</t>
+          <t>units_sold</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2000</v>
+        <v>79</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1997,12 +2296,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>audio array</t>
+          <t>nexlev</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>flipkart</t>
+          <t>bi worldwide</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2011,7 +2310,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>151</v>
+        <v>99</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -2030,7 +2329,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bi worldwide</t>
+          <t>pharmaeasy</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2039,9 +2338,37 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>182</v>
+        <v>16</v>
       </c>
       <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1p sales</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>units_sold</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>482</v>
+      </c>
+      <c r="F5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2421,11 +2748,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MISSING — no rows for audio array in sales for W30</t>
+          <t>MISSING — no rows for audio array in sales for W31</t>
         </is>
       </c>
     </row>
@@ -2441,11 +2768,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MISSING — no rows for nexlev in sales for W30</t>
+          <t>MISSING — no rows for nexlev in sales for W31</t>
         </is>
       </c>
     </row>
@@ -2461,11 +2788,11 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MISSING — no rows for tonor in sales for W30</t>
+          <t>MISSING — no rows for tonor in sales for W31</t>
         </is>
       </c>
     </row>
@@ -2481,11 +2808,11 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MISSING — no rows for white mulberry in sales for W30</t>
+          <t>MISSING — no rows for white mulberry in sales for W31</t>
         </is>
       </c>
     </row>
@@ -2501,11 +2828,11 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MISSING — no rows for audio array in inventory for W30</t>
+          <t>MISSING — no rows for audio array in inventory for W31</t>
         </is>
       </c>
     </row>
@@ -2521,11 +2848,11 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MISSING — no rows for nexlev in inventory for W30</t>
+          <t>MISSING — no rows for nexlev in inventory for W31</t>
         </is>
       </c>
     </row>
@@ -2541,11 +2868,11 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MISSING — no rows for tonor in inventory for W30</t>
+          <t>MISSING — no rows for tonor in inventory for W31</t>
         </is>
       </c>
     </row>
@@ -2561,11 +2888,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MISSING — no rows for white mulberry in inventory for W30</t>
+          <t>MISSING — no rows for white mulberry in inventory for W31</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4727,6 +5054,126 @@
         <v>937</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>31</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>audio array</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>3085</v>
+      </c>
+      <c r="F90" t="n">
+        <v>3085</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>31</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>fossil</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" t="n">
+        <v>5927</v>
+      </c>
+      <c r="F91" t="n">
+        <v>5927</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>31</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>nexlev</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>9522</v>
+      </c>
+      <c r="F92" t="n">
+        <v>9522</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>31</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>tonor</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>364</v>
+      </c>
+      <c r="F93" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>31</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>white mulberry</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>980</v>
+      </c>
+      <c r="F94" t="n">
+        <v>980</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>